<commit_message>
Reformat Q1B owner's equity statement to Divine Designs lecture layout.
Uses middle column for Add: Net income, right column for running totals, single/double underlines matching the sample format.

Co-authored-by: Reze13omb <Reze13omb@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/A1A_Q1_8571260_completed.xlsx
+++ b/A1A_Q1_8571260_completed.xlsx
@@ -7,18 +7,19 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4300" yWindow="7750" windowWidth="12770" windowHeight="8690" tabRatio="891" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1B Statements" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="input" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="input reference" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="income statement and owners ref" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="balance sheet ref" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2 Cole TB" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3 NI" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Adjusted TB" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1B OE Statement" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1B Statements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="input" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="input reference" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="income statement and owners ref" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="balance sheet ref" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2 Cole TB" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3 NI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4 Adjusted TB" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'income statement and owners ref'!$A$1:$I$50</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'balance sheet ref'!$A$1:$I$50</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'income statement and owners ref'!$A$1:$I$50</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'balance sheet ref'!$A$1:$I$50</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +32,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="mmmm\ d\,\ yyyy"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Arial"/>
       <sz val="10"/>
@@ -102,6 +103,11 @@
       <name val="Times New Roman"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -122,7 +128,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="41">
+  <borders count="43">
     <border>
       <left/>
       <right/>
@@ -607,11 +613,17 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <bottom style="double"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -844,6 +856,22 @@
     <xf numFmtId="3" fontId="13" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="12" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1211,10 +1239,135 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="116" t="inlineStr">
+        <is>
+          <t>GLOSS &amp; GLOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="116" t="inlineStr">
+        <is>
+          <t>Owner's Equity Statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="116" t="inlineStr">
+        <is>
+          <t>For the Month Ended September 30, 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="117" t="n"/>
+      <c r="B4" s="117" t="n"/>
+      <c r="C4" s="117" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="118" t="inlineStr">
+        <is>
+          <t>Owner's capital, September 1</t>
+        </is>
+      </c>
+      <c r="B6" s="118" t="n"/>
+      <c r="C6" s="119" t="n">
+        <v>57126</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="118" t="inlineStr">
+        <is>
+          <t>Add:</t>
+        </is>
+      </c>
+      <c r="B7" s="118" t="n"/>
+      <c r="C7" s="118" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Net income</t>
+        </is>
+      </c>
+      <c r="B8" s="120" t="n">
+        <v>55850</v>
+      </c>
+      <c r="C8" s="118" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="118" t="n"/>
+      <c r="B9" s="118" t="n"/>
+      <c r="C9" s="85" t="n">
+        <v>55850</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="118" t="n"/>
+      <c r="B10" s="118" t="n"/>
+      <c r="C10" s="85" t="n">
+        <v>112976</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="118" t="inlineStr">
+        <is>
+          <t>Less: Drawings</t>
+        </is>
+      </c>
+      <c r="B11" s="118" t="n"/>
+      <c r="C11" s="120" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="121" t="inlineStr">
+        <is>
+          <t>Owner's capital, September 30</t>
+        </is>
+      </c>
+      <c r="B12" s="118" t="n"/>
+      <c r="C12" s="122" t="n">
+        <v>106976</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="123" t="inlineStr">
+        <is>
+          <t>Note: There were no additional owner investments in September. Only Net income is shown under "Add:", matching the Divine Designs lecture format (middle column for addends; right column for running totals).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C89"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1757,12 +1910,106 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="110">
+        <f>==== Q1B Owner's Equity Statement (lecture / Divine Designs format) =====</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="116" t="inlineStr">
+        <is>
+          <t>GLOSS &amp; GLOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="116" t="inlineStr">
+        <is>
+          <t>Owner's Equity Statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="116" t="inlineStr">
+        <is>
+          <t>For the Month Ended September 30, 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="117" t="n"/>
+      <c r="B81" s="117" t="n"/>
+      <c r="C81" s="117" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="118" t="inlineStr">
+        <is>
+          <t>Owner's capital, September 1</t>
+        </is>
+      </c>
+      <c r="C83" s="119" t="n">
+        <v>57126</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="118" t="inlineStr">
+        <is>
+          <t>Add:</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Net income</t>
+        </is>
+      </c>
+      <c r="B85" s="120" t="n">
+        <v>55850</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="C86" s="85" t="n">
+        <v>55850</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="C87" s="85" t="n">
+        <v>112976</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="118" t="inlineStr">
+        <is>
+          <t>Less: Drawings</t>
+        </is>
+      </c>
+      <c r="C88" s="120" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="121" t="inlineStr">
+        <is>
+          <t>Owner's capital, September 30</t>
+        </is>
+      </c>
+      <c r="C89" s="122" t="n">
+        <v>106976</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A80:C80"/>
+    <mergeCell ref="A79:C79"/>
+    <mergeCell ref="A78:C78"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2159,7 +2406,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2297,7 +2544,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3025,7 +3272,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3590,7 +3837,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3792,7 +4039,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3935,7 +4182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>